<commit_message>
Added final versions of test suites 'perfect' and 'uniform'
</commit_message>
<xml_diff>
--- a/idea/preset_suites_descriptions.xlsx
+++ b/idea/preset_suites_descriptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni\practice\load-balancing-algorithms\idea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989A1FE4-9914-4ACD-8148-D6B0C5A4263C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3754C2F3-997F-4E48-8CCC-293D64F65475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1B073830-342D-45B6-9306-A000FEF79D6B}"/>
   </bookViews>
@@ -225,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -236,6 +236,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -577,7 +578,7 @@
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="5" t="s">
@@ -603,7 +604,7 @@
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>19</v>
       </c>
       <c r="E4" s="5" t="s">
@@ -819,6 +820,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="E10:E11"/>
     <mergeCell ref="E26:E27"/>
     <mergeCell ref="E28:E29"/>
     <mergeCell ref="E30:E31"/>
@@ -828,12 +835,6 @@
     <mergeCell ref="E20:E21"/>
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="E12:E13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Completed all presets Completed the results table
</commit_message>
<xml_diff>
--- a/idea/preset_suites_descriptions.xlsx
+++ b/idea/preset_suites_descriptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni\practice\load-balancing-algorithms\idea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{104467A6-FFAA-4212-8651-A9539CC3A508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394F23F1-04E3-4CD3-B4B8-E17F71485F56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1B073830-342D-45B6-9306-A000FEF79D6B}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>Uniform</t>
   </si>
@@ -136,12 +136,6 @@
   </si>
   <si>
     <t>churnBad</t>
-  </si>
-  <si>
-    <t>crashScenario</t>
-  </si>
-  <si>
-    <t>юниформ разброс запросов, разная стоимость, разные сервера: через 20 сек самый сильный сервер падает, через 20 сек после этого подключают замену чуть хуже, итого 60 сек</t>
   </si>
   <si>
     <t>stickyDefault</t>
@@ -267,15 +261,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -590,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AE2E0B6-6C5C-4976-B6CB-F6523495D256}">
-  <dimension ref="A1:AT27"/>
+  <dimension ref="A1:AT25"/>
   <sheetFormatPr defaultRowHeight="33.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="51.5703125" style="1" customWidth="1"/>
@@ -600,11 +594,11 @@
     <col min="6" max="6" width="13.5703125" customWidth="1"/>
     <col min="7" max="7" width="18.28515625" customWidth="1"/>
     <col min="8" max="8" width="15.5703125" customWidth="1"/>
-    <col min="19" max="19" width="9.140625" style="10"/>
-    <col min="25" max="25" width="9.140625" style="10"/>
-    <col min="31" max="31" width="9.140625" style="10"/>
-    <col min="37" max="37" width="9.140625" style="10"/>
-    <col min="43" max="43" width="9.140625" style="10"/>
+    <col min="19" max="19" width="9.140625" style="9"/>
+    <col min="25" max="25" width="9.140625" style="9"/>
+    <col min="31" max="31" width="9.140625" style="9"/>
+    <col min="37" max="37" width="9.140625" style="9"/>
+    <col min="43" max="43" width="9.140625" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:46" ht="42" customHeight="1" x14ac:dyDescent="0.5">
@@ -617,11 +611,11 @@
       <c r="E1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="S1" s="9"/>
-      <c r="Y1" s="9"/>
-      <c r="AE1" s="9"/>
-      <c r="AK1" s="9"/>
-      <c r="AQ1" s="9"/>
+      <c r="S1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="AE1" s="8"/>
+      <c r="AK1" s="8"/>
+      <c r="AQ1" s="8"/>
     </row>
     <row r="2" spans="1:46" ht="38.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
@@ -630,7 +624,7 @@
       <c r="D2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="12" t="s">
         <v>15</v>
       </c>
       <c r="F2" t="s">
@@ -647,9 +641,9 @@
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="6"/>
+      <c r="E3" s="12"/>
       <c r="K3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:46" ht="39.75" customHeight="1" x14ac:dyDescent="0.5">
@@ -659,7 +653,7 @@
       <c r="D4" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="12" t="s">
         <v>20</v>
       </c>
       <c r="F4" t="s">
@@ -689,7 +683,7 @@
       <c r="R4">
         <v>5</v>
       </c>
-      <c r="S4" s="10">
+      <c r="S4" s="9">
         <v>6</v>
       </c>
       <c r="T4">
@@ -707,7 +701,7 @@
       <c r="X4">
         <v>11</v>
       </c>
-      <c r="Y4" s="10">
+      <c r="Y4" s="9">
         <v>12</v>
       </c>
       <c r="Z4">
@@ -725,7 +719,7 @@
       <c r="AD4">
         <v>17</v>
       </c>
-      <c r="AE4" s="10">
+      <c r="AE4" s="9">
         <v>18</v>
       </c>
       <c r="AF4">
@@ -743,7 +737,7 @@
       <c r="AJ4">
         <v>23</v>
       </c>
-      <c r="AK4" s="10">
+      <c r="AK4" s="9">
         <v>24</v>
       </c>
       <c r="AL4">
@@ -761,7 +755,7 @@
       <c r="AP4">
         <v>29</v>
       </c>
-      <c r="AQ4" s="10">
+      <c r="AQ4" s="9">
         <v>30</v>
       </c>
     </row>
@@ -769,19 +763,19 @@
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="M5" s="8"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
-      <c r="R5" s="8"/>
-      <c r="S5" s="12"/>
-      <c r="T5" s="8"/>
-      <c r="U5" s="8"/>
-      <c r="V5" s="8"/>
-      <c r="W5" s="8"/>
-      <c r="X5" s="8"/>
+      <c r="E5" s="12"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="7"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="7"/>
     </row>
     <row r="6" spans="1:46" x14ac:dyDescent="0.5">
       <c r="A6" s="4" t="s">
@@ -790,7 +784,7 @@
       <c r="D6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="12" t="s">
         <v>21</v>
       </c>
       <c r="F6" t="s">
@@ -802,24 +796,24 @@
       <c r="H6" t="s">
         <v>29</v>
       </c>
-      <c r="M6" s="7"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7"/>
-      <c r="R6" s="7"/>
-      <c r="Y6" s="11"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="Y6" s="10"/>
     </row>
     <row r="7" spans="1:46" x14ac:dyDescent="0.5">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="T7" s="7"/>
-      <c r="U7" s="7"/>
-      <c r="V7" s="7"/>
-      <c r="W7" s="7"/>
-      <c r="X7" s="7"/>
+      <c r="E7" s="12"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
     </row>
     <row r="8" spans="1:46" x14ac:dyDescent="0.5">
       <c r="A8" s="4" t="s">
@@ -828,7 +822,7 @@
       <c r="D8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="12" t="s">
         <v>22</v>
       </c>
       <c r="F8" t="s">
@@ -840,31 +834,31 @@
       <c r="H8" t="s">
         <v>26</v>
       </c>
-      <c r="Z8" s="8"/>
-      <c r="AA8" s="8"/>
-      <c r="AB8" s="8"/>
-      <c r="AC8" s="8"/>
-      <c r="AD8" s="8"/>
-      <c r="AE8" s="12"/>
-      <c r="AF8" s="8"/>
-      <c r="AG8" s="8"/>
-      <c r="AH8" s="8"/>
-      <c r="AI8" s="8"/>
-      <c r="AJ8" s="8"/>
+      <c r="Z8" s="7"/>
+      <c r="AA8" s="7"/>
+      <c r="AB8" s="7"/>
+      <c r="AC8" s="7"/>
+      <c r="AD8" s="7"/>
+      <c r="AE8" s="11"/>
+      <c r="AF8" s="7"/>
+      <c r="AG8" s="7"/>
+      <c r="AH8" s="7"/>
+      <c r="AI8" s="7"/>
+      <c r="AJ8" s="7"/>
     </row>
     <row r="9" spans="1:46" x14ac:dyDescent="0.5">
-      <c r="E9" s="6"/>
-      <c r="Z9" s="7"/>
-      <c r="AA9" s="7"/>
-      <c r="AB9" s="7"/>
-      <c r="AC9" s="7"/>
-      <c r="AD9" s="7"/>
+      <c r="E9" s="12"/>
+      <c r="Z9" s="6"/>
+      <c r="AA9" s="6"/>
+      <c r="AB9" s="6"/>
+      <c r="AC9" s="6"/>
+      <c r="AD9" s="6"/>
     </row>
     <row r="10" spans="1:46" x14ac:dyDescent="0.5">
       <c r="D10" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="12" t="s">
         <v>23</v>
       </c>
       <c r="F10" t="s">
@@ -876,43 +870,43 @@
       <c r="H10" t="s">
         <v>26</v>
       </c>
-      <c r="AF10" s="7"/>
-      <c r="AG10" s="7"/>
-      <c r="AH10" s="7"/>
-      <c r="AI10" s="7"/>
-      <c r="AJ10" s="7"/>
+      <c r="AF10" s="6"/>
+      <c r="AG10" s="6"/>
+      <c r="AH10" s="6"/>
+      <c r="AI10" s="6"/>
+      <c r="AJ10" s="6"/>
     </row>
     <row r="11" spans="1:46" x14ac:dyDescent="0.5">
-      <c r="E11" s="6"/>
-      <c r="AL11" s="8"/>
-      <c r="AM11" s="8"/>
-      <c r="AN11" s="8"/>
-      <c r="AO11" s="8"/>
-      <c r="AP11" s="8"/>
-      <c r="AQ11" s="12"/>
-      <c r="AR11" s="8"/>
-      <c r="AS11" s="8"/>
-      <c r="AT11" s="8"/>
+      <c r="E11" s="12"/>
+      <c r="AL11" s="7"/>
+      <c r="AM11" s="7"/>
+      <c r="AN11" s="7"/>
+      <c r="AO11" s="7"/>
+      <c r="AP11" s="7"/>
+      <c r="AQ11" s="11"/>
+      <c r="AR11" s="7"/>
+      <c r="AS11" s="7"/>
+      <c r="AT11" s="7"/>
     </row>
     <row r="12" spans="1:46" x14ac:dyDescent="0.5">
       <c r="D12" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="AL12" s="7"/>
-      <c r="AM12" s="7"/>
-      <c r="AN12" s="7"/>
-      <c r="AO12" s="7"/>
-      <c r="AP12" s="7"/>
+      <c r="AL12" s="6"/>
+      <c r="AM12" s="6"/>
+      <c r="AN12" s="6"/>
+      <c r="AO12" s="6"/>
+      <c r="AP12" s="6"/>
     </row>
     <row r="13" spans="1:46" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="2"/>
-      <c r="E13" s="6"/>
+      <c r="E13" s="12"/>
     </row>
     <row r="14" spans="1:46" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
@@ -924,7 +918,7 @@
       <c r="D14" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="12" t="s">
         <v>33</v>
       </c>
     </row>
@@ -932,79 +926,67 @@
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="6"/>
+      <c r="E15" s="12"/>
     </row>
     <row r="16" spans="1:46" x14ac:dyDescent="0.5">
       <c r="D16" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E16" s="6" t="s">
-        <v>41</v>
+      <c r="E16" s="12" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E17" s="6"/>
+      <c r="E17" s="12"/>
     </row>
     <row r="18" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>42</v>
+      <c r="E18" s="12" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E19" s="6"/>
+      <c r="E19" s="12"/>
     </row>
     <row r="20" spans="4:5" x14ac:dyDescent="0.5">
       <c r="D20" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="4:5" x14ac:dyDescent="0.5">
+      <c r="E21" s="12"/>
+    </row>
+    <row r="22" spans="4:5" x14ac:dyDescent="0.5">
+      <c r="D22" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="23" spans="4:5" x14ac:dyDescent="0.5">
+      <c r="E23" s="12"/>
+    </row>
+    <row r="24" spans="4:5" x14ac:dyDescent="0.5">
+      <c r="D24" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="12" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E21" s="6"/>
-    </row>
-    <row r="22" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="D22" t="s">
-        <v>37</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="23" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E23" s="6"/>
-    </row>
-    <row r="24" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="D24" t="s">
-        <v>39</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="25" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E25" s="6"/>
-    </row>
-    <row r="26" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="D26" t="s">
-        <v>40</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="4:5" x14ac:dyDescent="0.5">
-      <c r="E27" s="6"/>
+      <c r="E25" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
     <mergeCell ref="E22:E23"/>
     <mergeCell ref="E24:E25"/>
-    <mergeCell ref="E26:E27"/>
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="E18:E19"/>

</xml_diff>